<commit_message>
mouse params + gui path location
</commit_message>
<xml_diff>
--- a/Params/Mouse_Room_Params.xlsx
+++ b/Params/Mouse_Room_Params.xlsx
@@ -1117,7 +1117,28 @@
         <v>0.8</v>
       </c>
       <c r="AK6" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL6" t="str">
+        <v>Fiber</v>
+      </c>
+      <c r="AN6" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP6" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR6" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS6" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU6" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV6" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="7">
@@ -1227,7 +1248,28 @@
         <v>0.8</v>
       </c>
       <c r="AK7" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL7" t="str">
+        <v>Fiber</v>
+      </c>
+      <c r="AN7" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP7" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR7" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS7" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU7" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV7" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="8">
@@ -1337,7 +1379,31 @@
         <v>0.8</v>
       </c>
       <c r="AK8" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL8" t="str">
+        <v>Zapit</v>
+      </c>
+      <c r="AM8" t="str">
+        <v>1</v>
+      </c>
+      <c r="AN8" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP8" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR8" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS8" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU8" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV8" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="9">
@@ -1447,7 +1513,31 @@
         <v>0.8</v>
       </c>
       <c r="AK9" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL9" t="str">
+        <v>Zapit</v>
+      </c>
+      <c r="AM9" t="str">
+        <v>1</v>
+      </c>
+      <c r="AN9" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP9" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR9" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS9" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU9" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV9" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="10">
@@ -1557,7 +1647,31 @@
         <v>0.8</v>
       </c>
       <c r="AK10" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL10" t="str">
+        <v>Zapit</v>
+      </c>
+      <c r="AM10" t="str">
+        <v>1</v>
+      </c>
+      <c r="AN10" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP10" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR10" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS10" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU10" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV10" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="11">
@@ -1667,7 +1781,31 @@
         <v>0.8</v>
       </c>
       <c r="AK11" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL11" t="str">
+        <v>Zapit</v>
+      </c>
+      <c r="AM11" t="str">
+        <v>1</v>
+      </c>
+      <c r="AN11" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP11" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR11" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS11" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU11" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV11" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="12">
@@ -1777,7 +1915,31 @@
         <v>0.8</v>
       </c>
       <c r="AK12" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL12" t="str">
+        <v>Zapit</v>
+      </c>
+      <c r="AM12" t="str">
+        <v>1</v>
+      </c>
+      <c r="AN12" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP12" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR12" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS12" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU12" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV12" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="13">
@@ -1887,7 +2049,28 @@
         <v>0.8</v>
       </c>
       <c r="AK13" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL13" t="str">
+        <v>Fiber</v>
+      </c>
+      <c r="AN13" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP13" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR13" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS13" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU13" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV13" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="14">
@@ -1997,7 +2180,28 @@
         <v>0.8</v>
       </c>
       <c r="AK14" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL14" t="str">
+        <v>Fiber</v>
+      </c>
+      <c r="AN14" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP14" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR14" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS14" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU14" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV14" t="str">
+        <v>PPC</v>
       </c>
     </row>
     <row r="15">
@@ -2107,7 +2311,28 @@
         <v>0.8</v>
       </c>
       <c r="AK15" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
+      </c>
+      <c r="AL15" t="str">
+        <v>Fiber</v>
+      </c>
+      <c r="AN15" t="str">
+        <v>30</v>
+      </c>
+      <c r="AP15" t="str">
+        <v>Sound</v>
+      </c>
+      <c r="AR15" t="str">
+        <v>Feedback</v>
+      </c>
+      <c r="AS15" t="str">
+        <v>Inter_Trial_Interval</v>
+      </c>
+      <c r="AU15" t="str">
+        <v>Bilateral</v>
+      </c>
+      <c r="AV15" t="str">
+        <v>PPC</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new batch -> lick to release
</commit_message>
<xml_diff>
--- a/Params/Mouse_Room_Params.xlsx
+++ b/Params/Mouse_Room_Params.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="109">
   <si>
     <t>Subject</t>
   </si>
@@ -196,34 +196,34 @@
     <t>Fixed</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>1.75</t>
+  </si>
+  <si>
+    <t>0.8</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
     <t>300</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>1.75</t>
-  </si>
-  <si>
-    <t>0.8</t>
-  </si>
-  <si>
-    <t>0.5</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>82</t>
   </si>
   <si>
     <t>20</t>
@@ -348,13 +348,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -365,7 +371,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -377,7 +390,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -385,7 +398,13 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
   </cellXfs>
@@ -693,55 +712,55 @@
   <dimension ref="A1:AW25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="37" max="37" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="38" max="38" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="39" max="39" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="40" max="40" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="41" max="41" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="42" max="42" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="43" max="43" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="44" max="44" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="45" max="45" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="46" max="46" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="47" max="47" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="48" max="48" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="49" max="49" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="44" max="44" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="45" max="45" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="46" max="46" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="47" max="47" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="48" max="48" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="49" max="49" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -784,7 +803,7 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
@@ -931,62 +950,62 @@
       <c r="M2" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="N2" s="2">
+        <v>300</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="R2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="R2" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="S2" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U2" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V2" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Z2" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB2" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC2" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD2" s="1" t="s">
+      <c r="AE2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE2" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG2" s="1" t="s">
         <v>52</v>
@@ -995,10 +1014,10 @@
         <v>70</v>
       </c>
       <c r="AI2" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ2" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK2" s="1" t="s">
         <v>56</v>
@@ -1054,62 +1073,62 @@
       <c r="M3" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="N3" s="2">
+        <v>300</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P3" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="R3" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="S3" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U3" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V3" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y3" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z3" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD3" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB3" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD3" s="1" t="s">
+      <c r="AE3" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE3" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG3" s="1" t="s">
         <v>52</v>
@@ -1118,10 +1137,10 @@
         <v>70</v>
       </c>
       <c r="AI3" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ3" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK3" s="1" t="s">
         <v>56</v>
@@ -1177,62 +1196,62 @@
       <c r="M4" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="N4" s="2">
+        <v>300</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O4" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="R4" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="R4" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="S4" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U4" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U4" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V4" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y4" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z4" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA4" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB4" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD4" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB4" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC4" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD4" s="1" t="s">
+      <c r="AE4" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE4" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF4" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG4" s="1" t="s">
         <v>52</v>
@@ -1241,10 +1260,10 @@
         <v>70</v>
       </c>
       <c r="AI4" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK4" s="1" t="s">
         <v>56</v>
@@ -1300,41 +1319,41 @@
       <c r="M5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="N5" s="2">
+        <v>300</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O5" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q5" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S5" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U5" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V5" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X5" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y5" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z5" s="1" t="s">
         <v>55</v>
@@ -1343,19 +1362,19 @@
         <v>78</v>
       </c>
       <c r="AB5" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AC5" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AD5" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE5" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE5" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF5" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG5" s="1" t="s">
         <v>52</v>
@@ -1367,7 +1386,7 @@
         <v>55</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK5" s="1" t="s">
         <v>56</v>
@@ -1377,7 +1396,7 @@
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO5" s="1"/>
       <c r="AP5" s="1" t="s">
@@ -1437,62 +1456,62 @@
       <c r="M6" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="3">
         <v>150</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S6" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T6" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U6" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U6" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V6" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y6" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z6" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC6" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD6" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB6" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD6" s="1" t="s">
+      <c r="AE6" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE6" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG6" s="1" t="s">
         <v>52</v>
@@ -1501,10 +1520,10 @@
         <v>70</v>
       </c>
       <c r="AI6" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK6" s="1" t="s">
         <v>56</v>
@@ -1514,7 +1533,7 @@
       </c>
       <c r="AM6" s="1"/>
       <c r="AN6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO6" s="1"/>
       <c r="AP6" s="1" t="s">
@@ -1574,62 +1593,62 @@
       <c r="M7" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="3">
         <v>150</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U7" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U7" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V7" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z7" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA7" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC7" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD7" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB7" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC7" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD7" s="1" t="s">
+      <c r="AE7" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE7" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF7" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG7" s="1" t="s">
         <v>52</v>
@@ -1638,10 +1657,10 @@
         <v>70</v>
       </c>
       <c r="AI7" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ7" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK7" s="1" t="s">
         <v>56</v>
@@ -1651,7 +1670,7 @@
       </c>
       <c r="AM7" s="1"/>
       <c r="AN7" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO7" s="1"/>
       <c r="AP7" s="1" t="s">
@@ -1711,62 +1730,62 @@
       <c r="M8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="3">
         <v>150</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S8" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T8" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U8" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U8" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V8" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z8" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC8" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD8" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB8" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC8" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD8" s="1" t="s">
+      <c r="AE8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE8" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF8" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG8" s="1" t="s">
         <v>52</v>
@@ -1775,10 +1794,10 @@
         <v>70</v>
       </c>
       <c r="AI8" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK8" s="1" t="s">
         <v>56</v>
@@ -1787,10 +1806,10 @@
         <v>91</v>
       </c>
       <c r="AM8" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AN8" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO8" s="1"/>
       <c r="AP8" s="1" t="s">
@@ -1850,62 +1869,62 @@
       <c r="M9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="3">
         <v>150</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S9" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T9" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U9" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U9" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V9" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X9" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z9" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA9" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD9" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB9" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD9" s="1" t="s">
+      <c r="AE9" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE9" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF9" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG9" s="1" t="s">
         <v>52</v>
@@ -1914,10 +1933,10 @@
         <v>70</v>
       </c>
       <c r="AI9" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ9" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK9" s="1" t="s">
         <v>56</v>
@@ -1926,10 +1945,10 @@
         <v>91</v>
       </c>
       <c r="AM9" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AN9" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO9" s="1"/>
       <c r="AP9" s="1" t="s">
@@ -1989,62 +2008,62 @@
       <c r="M10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="3">
         <v>150</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U10" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U10" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X10" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y10" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z10" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC10" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD10" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB10" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC10" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD10" s="1" t="s">
+      <c r="AE10" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE10" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF10" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG10" s="1" t="s">
         <v>52</v>
@@ -2053,10 +2072,10 @@
         <v>70</v>
       </c>
       <c r="AI10" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ10" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK10" s="1" t="s">
         <v>56</v>
@@ -2065,10 +2084,10 @@
         <v>91</v>
       </c>
       <c r="AM10" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AN10" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO10" s="1"/>
       <c r="AP10" s="1" t="s">
@@ -2128,62 +2147,62 @@
       <c r="M11" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="3">
         <v>150</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S11" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U11" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U11" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V11" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X11" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y11" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z11" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD11" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC11" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD11" s="1" t="s">
+      <c r="AE11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE11" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF11" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG11" s="1" t="s">
         <v>52</v>
@@ -2192,10 +2211,10 @@
         <v>70</v>
       </c>
       <c r="AI11" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ11" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK11" s="1" t="s">
         <v>56</v>
@@ -2204,10 +2223,10 @@
         <v>91</v>
       </c>
       <c r="AM11" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AN11" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO11" s="1"/>
       <c r="AP11" s="1" t="s">
@@ -2267,62 +2286,62 @@
       <c r="M12" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="3">
         <v>150</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S12" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T12" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U12" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V12" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X12" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y12" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z12" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA12" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC12" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD12" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB12" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC12" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD12" s="1" t="s">
+      <c r="AE12" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE12" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF12" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG12" s="1" t="s">
         <v>52</v>
@@ -2331,10 +2350,10 @@
         <v>70</v>
       </c>
       <c r="AI12" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ12" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK12" s="1" t="s">
         <v>56</v>
@@ -2343,10 +2362,10 @@
         <v>91</v>
       </c>
       <c r="AM12" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AN12" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO12" s="1"/>
       <c r="AP12" s="1" t="s">
@@ -2406,62 +2425,62 @@
       <c r="M13" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="3">
         <v>150</v>
       </c>
       <c r="O13" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S13" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U13" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U13" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V13" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X13" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y13" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z13" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA13" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD13" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB13" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC13" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD13" s="1" t="s">
+      <c r="AE13" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE13" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF13" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG13" s="1" t="s">
         <v>52</v>
@@ -2470,10 +2489,10 @@
         <v>70</v>
       </c>
       <c r="AI13" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ13" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK13" s="1" t="s">
         <v>56</v>
@@ -2483,7 +2502,7 @@
       </c>
       <c r="AM13" s="1"/>
       <c r="AN13" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO13" s="1"/>
       <c r="AP13" s="1" t="s">
@@ -2543,62 +2562,62 @@
       <c r="M14" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="3">
         <v>150</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S14" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T14" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U14" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U14" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V14" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X14" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y14" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z14" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA14" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB14" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC14" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD14" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB14" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC14" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD14" s="1" t="s">
+      <c r="AE14" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE14" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF14" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG14" s="1" t="s">
         <v>52</v>
@@ -2607,10 +2626,10 @@
         <v>70</v>
       </c>
       <c r="AI14" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ14" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK14" s="1" t="s">
         <v>56</v>
@@ -2620,7 +2639,7 @@
       </c>
       <c r="AM14" s="1"/>
       <c r="AN14" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO14" s="1"/>
       <c r="AP14" s="1" t="s">
@@ -2680,62 +2699,62 @@
       <c r="M15" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="3">
         <v>150</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>52</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S15" s="1" t="s">
         <v>56</v>
       </c>
       <c r="T15" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U15" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U15" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V15" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X15" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y15" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Z15" s="1" t="s">
         <v>55</v>
       </c>
       <c r="AA15" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB15" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD15" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB15" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC15" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD15" s="1" t="s">
+      <c r="AE15" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE15" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF15" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG15" s="1" t="s">
         <v>52</v>
@@ -2744,10 +2763,10 @@
         <v>70</v>
       </c>
       <c r="AI15" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ15" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK15" s="1" t="s">
         <v>56</v>
@@ -2757,7 +2776,7 @@
       </c>
       <c r="AM15" s="1"/>
       <c r="AN15" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO15" s="1"/>
       <c r="AP15" s="1" t="s">
@@ -2787,7 +2806,7 @@
         <v>50</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1" t="s">
@@ -2817,17 +2836,17 @@
       <c r="M16" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N16" s="1" t="s">
+      <c r="N16" s="2">
+        <v>300</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P16" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O16" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q16" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R16" s="1" t="s">
         <v>55</v>
@@ -2836,43 +2855,43 @@
         <v>56</v>
       </c>
       <c r="T16" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U16" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U16" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V16" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z16" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA16" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB16" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y16" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z16" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA16" s="1" t="s">
+      <c r="AC16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD16" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB16" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC16" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD16" s="1" t="s">
+      <c r="AE16" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE16" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF16" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG16" s="1" t="s">
         <v>52</v>
@@ -2881,10 +2900,10 @@
         <v>70</v>
       </c>
       <c r="AI16" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ16" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK16" s="1" t="s">
         <v>56</v>
@@ -2894,7 +2913,7 @@
       </c>
       <c r="AM16" s="1"/>
       <c r="AN16" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO16" s="1"/>
       <c r="AP16" s="1" t="s">
@@ -2924,7 +2943,7 @@
         <v>50</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
@@ -2954,17 +2973,17 @@
       <c r="M17" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N17" s="1" t="s">
+      <c r="N17" s="2">
+        <v>300</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P17" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O17" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P17" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q17" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R17" s="1" t="s">
         <v>55</v>
@@ -2973,43 +2992,43 @@
         <v>56</v>
       </c>
       <c r="T17" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U17" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U17" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V17" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W17" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X17" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y17" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z17" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA17" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB17" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y17" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z17" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA17" s="1" t="s">
+      <c r="AC17" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD17" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB17" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC17" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD17" s="1" t="s">
+      <c r="AE17" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE17" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF17" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG17" s="1" t="s">
         <v>52</v>
@@ -3018,10 +3037,10 @@
         <v>70</v>
       </c>
       <c r="AI17" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ17" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK17" s="1" t="s">
         <v>56</v>
@@ -3031,7 +3050,7 @@
       </c>
       <c r="AM17" s="1"/>
       <c r="AN17" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO17" s="1"/>
       <c r="AP17" s="1" t="s">
@@ -3061,7 +3080,7 @@
         <v>50</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
@@ -3091,17 +3110,17 @@
       <c r="M18" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N18" s="1" t="s">
+      <c r="N18" s="2">
+        <v>300</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P18" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O18" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P18" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q18" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R18" s="1" t="s">
         <v>55</v>
@@ -3110,43 +3129,43 @@
         <v>56</v>
       </c>
       <c r="T18" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U18" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U18" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V18" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W18" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X18" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y18" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z18" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA18" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB18" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y18" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z18" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA18" s="1" t="s">
+      <c r="AC18" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD18" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB18" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC18" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD18" s="1" t="s">
+      <c r="AE18" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE18" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF18" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG18" s="1" t="s">
         <v>52</v>
@@ -3155,10 +3174,10 @@
         <v>70</v>
       </c>
       <c r="AI18" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ18" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK18" s="1" t="s">
         <v>56</v>
@@ -3168,7 +3187,7 @@
       </c>
       <c r="AM18" s="1"/>
       <c r="AN18" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO18" s="1"/>
       <c r="AP18" s="1" t="s">
@@ -3198,7 +3217,7 @@
         <v>50</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1" t="s">
@@ -3228,17 +3247,17 @@
       <c r="M19" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N19" s="1" t="s">
+      <c r="N19" s="2">
+        <v>300</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P19" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O19" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q19" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R19" s="1" t="s">
         <v>55</v>
@@ -3247,43 +3266,43 @@
         <v>56</v>
       </c>
       <c r="T19" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U19" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U19" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V19" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W19" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X19" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y19" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z19" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB19" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y19" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z19" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA19" s="1" t="s">
+      <c r="AC19" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD19" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB19" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC19" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD19" s="1" t="s">
+      <c r="AE19" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE19" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF19" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG19" s="1" t="s">
         <v>52</v>
@@ -3292,10 +3311,10 @@
         <v>70</v>
       </c>
       <c r="AI19" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ19" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK19" s="1" t="s">
         <v>56</v>
@@ -3305,7 +3324,7 @@
       </c>
       <c r="AM19" s="1"/>
       <c r="AN19" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO19" s="1"/>
       <c r="AP19" s="1" t="s">
@@ -3335,7 +3354,7 @@
         <v>50</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1" t="s">
@@ -3365,17 +3384,17 @@
       <c r="M20" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N20" s="1" t="s">
+      <c r="N20" s="2">
+        <v>300</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P20" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O20" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P20" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q20" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R20" s="1" t="s">
         <v>55</v>
@@ -3384,43 +3403,43 @@
         <v>56</v>
       </c>
       <c r="T20" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U20" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U20" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V20" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W20" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z20" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA20" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB20" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y20" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z20" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA20" s="1" t="s">
+      <c r="AC20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD20" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB20" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC20" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD20" s="1" t="s">
+      <c r="AE20" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE20" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF20" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG20" s="1" t="s">
         <v>52</v>
@@ -3429,10 +3448,10 @@
         <v>70</v>
       </c>
       <c r="AI20" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ20" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK20" s="1" t="s">
         <v>56</v>
@@ -3442,7 +3461,7 @@
       </c>
       <c r="AM20" s="1"/>
       <c r="AN20" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO20" s="1"/>
       <c r="AP20" s="1" t="s">
@@ -3472,7 +3491,7 @@
         <v>50</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
@@ -3502,17 +3521,17 @@
       <c r="M21" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N21" s="1" t="s">
+      <c r="N21" s="2">
+        <v>300</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P21" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O21" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P21" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q21" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R21" s="1" t="s">
         <v>55</v>
@@ -3521,43 +3540,43 @@
         <v>56</v>
       </c>
       <c r="T21" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U21" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U21" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V21" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W21" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X21" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y21" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z21" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA21" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB21" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y21" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z21" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA21" s="1" t="s">
+      <c r="AC21" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD21" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB21" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC21" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD21" s="1" t="s">
+      <c r="AE21" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE21" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF21" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG21" s="1" t="s">
         <v>52</v>
@@ -3566,10 +3585,10 @@
         <v>70</v>
       </c>
       <c r="AI21" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ21" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK21" s="1" t="s">
         <v>56</v>
@@ -3579,7 +3598,7 @@
       </c>
       <c r="AM21" s="1"/>
       <c r="AN21" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO21" s="1"/>
       <c r="AP21" s="1" t="s">
@@ -3609,7 +3628,7 @@
         <v>50</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1" t="s">
@@ -3639,17 +3658,17 @@
       <c r="M22" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N22" s="1" t="s">
+      <c r="N22" s="2">
+        <v>300</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P22" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O22" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="P22" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q22" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R22" s="1" t="s">
         <v>55</v>
@@ -3658,43 +3677,43 @@
         <v>56</v>
       </c>
       <c r="T22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U22" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U22" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V22" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X22" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y22" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z22" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA22" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB22" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y22" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z22" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA22" s="1" t="s">
+      <c r="AC22" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD22" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB22" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC22" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD22" s="1" t="s">
+      <c r="AE22" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE22" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF22" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG22" s="1" t="s">
         <v>52</v>
@@ -3703,10 +3722,10 @@
         <v>70</v>
       </c>
       <c r="AI22" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ22" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK22" s="1" t="s">
         <v>56</v>
@@ -3716,7 +3735,7 @@
       </c>
       <c r="AM22" s="1"/>
       <c r="AN22" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO22" s="1"/>
       <c r="AP22" s="1" t="s">
@@ -3746,7 +3765,7 @@
         <v>50</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1" t="s">
@@ -3776,17 +3795,17 @@
       <c r="M23" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N23" s="1" t="s">
+      <c r="N23" s="2">
+        <v>300</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P23" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O23" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q23" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R23" s="1" t="s">
         <v>55</v>
@@ -3795,43 +3814,43 @@
         <v>56</v>
       </c>
       <c r="T23" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U23" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U23" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V23" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W23" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X23" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y23" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z23" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA23" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB23" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y23" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z23" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA23" s="1" t="s">
+      <c r="AC23" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD23" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB23" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC23" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD23" s="1" t="s">
+      <c r="AE23" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE23" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF23" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG23" s="1" t="s">
         <v>52</v>
@@ -3840,10 +3859,10 @@
         <v>70</v>
       </c>
       <c r="AI23" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ23" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK23" s="1" t="s">
         <v>56</v>
@@ -3853,7 +3872,7 @@
       </c>
       <c r="AM23" s="1"/>
       <c r="AN23" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO23" s="1"/>
       <c r="AP23" s="1" t="s">
@@ -3883,7 +3902,7 @@
         <v>50</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1" t="s">
@@ -3913,17 +3932,17 @@
       <c r="M24" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N24" s="1" t="s">
+      <c r="N24" s="2">
+        <v>300</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P24" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O24" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P24" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q24" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R24" s="1" t="s">
         <v>55</v>
@@ -3932,43 +3951,43 @@
         <v>56</v>
       </c>
       <c r="T24" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U24" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U24" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V24" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W24" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z24" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA24" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB24" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y24" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z24" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA24" s="1" t="s">
+      <c r="AC24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD24" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB24" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC24" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD24" s="1" t="s">
+      <c r="AE24" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE24" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF24" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG24" s="1" t="s">
         <v>52</v>
@@ -3977,10 +3996,10 @@
         <v>70</v>
       </c>
       <c r="AI24" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ24" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK24" s="1" t="s">
         <v>56</v>
@@ -3990,7 +4009,7 @@
       </c>
       <c r="AM24" s="1"/>
       <c r="AN24" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO24" s="1"/>
       <c r="AP24" s="1" t="s">
@@ -4020,7 +4039,7 @@
         <v>50</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1" t="s">
@@ -4050,17 +4069,17 @@
       <c r="M25" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="N25" s="1" t="s">
+      <c r="N25" s="2">
+        <v>300</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P25" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="O25" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="P25" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="Q25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="R25" s="1" t="s">
         <v>55</v>
@@ -4069,43 +4088,43 @@
         <v>56</v>
       </c>
       <c r="T25" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="U25" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="U25" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="V25" s="1" t="s">
         <v>56</v>
       </c>
       <c r="W25" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X25" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y25" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Z25" s="2">
+        <v>2</v>
+      </c>
+      <c r="AA25" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB25" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Y25" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Z25" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA25" s="1" t="s">
+      <c r="AC25" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD25" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AB25" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC25" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD25" s="1" t="s">
+      <c r="AE25" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AE25" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="AF25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG25" s="1" t="s">
         <v>52</v>
@@ -4114,10 +4133,10 @@
         <v>70</v>
       </c>
       <c r="AI25" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AJ25" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AK25" s="1" t="s">
         <v>56</v>
@@ -4127,7 +4146,7 @@
       </c>
       <c r="AM25" s="1"/>
       <c r="AN25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AO25" s="1"/>
       <c r="AP25" s="1" t="s">

</xml_diff>

<commit_message>
new cohort --> full task
</commit_message>
<xml_diff>
--- a/Params/Mouse_Room_Params.xlsx
+++ b/Params/Mouse_Room_Params.xlsx
@@ -2342,7 +2342,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C16" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E16" t="str">
         <v>TRUE</v>
@@ -2354,7 +2354,7 @@
         <v>WN</v>
       </c>
       <c r="H16" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I16" t="str">
         <v>FALSE</v>
@@ -2473,7 +2473,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C17" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E17" t="str">
         <v>TRUE</v>
@@ -2485,7 +2485,7 @@
         <v>WN</v>
       </c>
       <c r="H17" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I17" t="str">
         <v>FALSE</v>
@@ -2604,7 +2604,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C18" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E18" t="str">
         <v>TRUE</v>
@@ -2616,7 +2616,7 @@
         <v>WN</v>
       </c>
       <c r="H18" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I18" t="str">
         <v>FALSE</v>
@@ -2735,7 +2735,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C19" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E19" t="str">
         <v>TRUE</v>
@@ -2747,7 +2747,7 @@
         <v>WN</v>
       </c>
       <c r="H19" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I19" t="str">
         <v>FALSE</v>
@@ -2866,7 +2866,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C20" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E20" t="str">
         <v>TRUE</v>
@@ -2878,7 +2878,7 @@
         <v>WN</v>
       </c>
       <c r="H20" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I20" t="str">
         <v>FALSE</v>
@@ -2997,7 +2997,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C21" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E21" t="str">
         <v>TRUE</v>
@@ -3009,7 +3009,7 @@
         <v>WN</v>
       </c>
       <c r="H21" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I21" t="str">
         <v>FALSE</v>
@@ -3128,7 +3128,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C22" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E22" t="str">
         <v>TRUE</v>
@@ -3140,7 +3140,7 @@
         <v>WN</v>
       </c>
       <c r="H22" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I22" t="str">
         <v>FALSE</v>
@@ -3259,7 +3259,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C23" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E23" t="str">
         <v>TRUE</v>
@@ -3271,7 +3271,7 @@
         <v>WN</v>
       </c>
       <c r="H23" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I23" t="str">
         <v>FALSE</v>
@@ -3390,7 +3390,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C24" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E24" t="str">
         <v>TRUE</v>
@@ -3402,7 +3402,7 @@
         <v>WN</v>
       </c>
       <c r="H24" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I24" t="str">
         <v>FALSE</v>
@@ -3521,7 +3521,7 @@
         <v>SOUND_CAT</v>
       </c>
       <c r="C25" t="str">
-        <v>Three_And_Three</v>
+        <v>Full_Task_Cont</v>
       </c>
       <c r="E25" t="str">
         <v>TRUE</v>

</xml_diff>

<commit_message>
mouse params updated -- 3 zapit
</commit_message>
<xml_diff>
--- a/Params/Mouse_Room_Params.xlsx
+++ b/Params/Mouse_Room_Params.xlsx
@@ -2345,7 +2345,7 @@
         <v>Full_Task_Cont</v>
       </c>
       <c r="E16" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="F16" t="str">
         <v>Uniform</v>
@@ -2375,7 +2375,7 @@
         <v>150</v>
       </c>
       <c r="O16" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="P16" t="str">
         <v>1</v>
@@ -2384,7 +2384,7 @@
         <v>30</v>
       </c>
       <c r="R16" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="str">
         <v>FALSE</v>
@@ -2476,7 +2476,7 @@
         <v>Full_Task_Cont</v>
       </c>
       <c r="E17" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="F17" t="str">
         <v>Uniform</v>
@@ -2515,7 +2515,7 @@
         <v>30</v>
       </c>
       <c r="R17" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" t="str">
         <v>FALSE</v>
@@ -2703,10 +2703,10 @@
         <v>0.8</v>
       </c>
       <c r="AK18" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="AL18" t="str">
-        <v>Fiber</v>
+        <v>Zapit</v>
       </c>
       <c r="AN18" t="str">
         <v>30</v>
@@ -2768,7 +2768,7 @@
         <v>150</v>
       </c>
       <c r="O19" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="P19" t="str">
         <v>1</v>
@@ -2777,7 +2777,7 @@
         <v>30</v>
       </c>
       <c r="R19" t="str">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="S19" t="str">
         <v>FALSE</v>
@@ -2869,7 +2869,7 @@
         <v>Full_Task_Cont</v>
       </c>
       <c r="E20" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="F20" t="str">
         <v>Uniform</v>
@@ -2899,7 +2899,7 @@
         <v>150</v>
       </c>
       <c r="O20" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="P20" t="str">
         <v>1</v>
@@ -2908,7 +2908,7 @@
         <v>30</v>
       </c>
       <c r="R20" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="str">
         <v>FALSE</v>
@@ -3131,7 +3131,7 @@
         <v>Full_Task_Cont</v>
       </c>
       <c r="E22" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="F22" t="str">
         <v>Uniform</v>
@@ -3161,7 +3161,7 @@
         <v>150</v>
       </c>
       <c r="O22" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="P22" t="str">
         <v>1</v>
@@ -3170,7 +3170,7 @@
         <v>30</v>
       </c>
       <c r="R22" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S22" t="str">
         <v>FALSE</v>
@@ -3358,10 +3358,10 @@
         <v>0.8</v>
       </c>
       <c r="AK23" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="AL23" t="str">
-        <v>Fiber</v>
+        <v>Zapit</v>
       </c>
       <c r="AN23" t="str">
         <v>30</v>
@@ -3524,7 +3524,7 @@
         <v>Full_Task_Cont</v>
       </c>
       <c r="E25" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="F25" t="str">
         <v>Uniform</v>
@@ -3551,7 +3551,7 @@
         <v>Fixed</v>
       </c>
       <c r="N25" t="str">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="O25" t="str">
         <v>TRUE</v>
@@ -3563,7 +3563,7 @@
         <v>30</v>
       </c>
       <c r="R25" t="str">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="S25" t="str">
         <v>FALSE</v>
@@ -3620,10 +3620,10 @@
         <v>0.8</v>
       </c>
       <c r="AK25" t="str">
-        <v>FALSE</v>
+        <v>TRUE</v>
       </c>
       <c r="AL25" t="str">
-        <v>Fiber</v>
+        <v>Zapit</v>
       </c>
       <c r="AN25" t="str">
         <v>30</v>

</xml_diff>

<commit_message>
first batch asym_right (hard a)
</commit_message>
<xml_diff>
--- a/Params/Mouse_Room_Params.xlsx
+++ b/Params/Mouse_Room_Params.xlsx
@@ -1026,7 +1026,7 @@
         <v>FALSE</v>
       </c>
       <c r="F6" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G6" t="str">
         <v>WN</v>
@@ -1160,7 +1160,7 @@
         <v>FALSE</v>
       </c>
       <c r="F7" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G7" t="str">
         <v>WN</v>
@@ -1294,7 +1294,7 @@
         <v>FALSE</v>
       </c>
       <c r="F8" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G8" t="str">
         <v>WN</v>
@@ -1428,7 +1428,7 @@
         <v>FALSE</v>
       </c>
       <c r="F9" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G9" t="str">
         <v>WN</v>
@@ -1562,7 +1562,7 @@
         <v>FALSE</v>
       </c>
       <c r="F10" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G10" t="str">
         <v>WN</v>
@@ -1696,7 +1696,7 @@
         <v>FALSE</v>
       </c>
       <c r="F11" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G11" t="str">
         <v>WN</v>
@@ -1830,7 +1830,7 @@
         <v>FALSE</v>
       </c>
       <c r="F12" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G12" t="str">
         <v>WN</v>
@@ -2098,7 +2098,7 @@
         <v>FALSE</v>
       </c>
       <c r="F14" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G14" t="str">
         <v>WN</v>
@@ -2232,7 +2232,7 @@
         <v>FALSE</v>
       </c>
       <c r="F15" t="str">
-        <v>Asym_Left</v>
+        <v>Asym_Right</v>
       </c>
       <c r="G15" t="str">
         <v>WN</v>

</xml_diff>

<commit_message>
zapit off for after opto washing
</commit_message>
<xml_diff>
--- a/Params/Mouse_Room_Params.xlsx
+++ b/Params/Mouse_Room_Params.xlsx
@@ -2232,7 +2232,7 @@
         <v>FALSE</v>
       </c>
       <c r="F15" t="str">
-        <v>Asym_Right</v>
+        <v>Asym_Left</v>
       </c>
       <c r="G15" t="str">
         <v>WN</v>
@@ -2459,7 +2459,7 @@
         <v>0.8</v>
       </c>
       <c r="AK16" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="AL16" t="str">
         <v>Zapit</v>
@@ -2593,7 +2593,7 @@
         <v>0.8</v>
       </c>
       <c r="AK17" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="AL17" t="str">
         <v>Zapit</v>
@@ -2727,7 +2727,7 @@
         <v>0.8</v>
       </c>
       <c r="AK18" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="AL18" t="str">
         <v>Zapit</v>
@@ -2995,7 +2995,7 @@
         <v>0.8</v>
       </c>
       <c r="AK20" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="AL20" t="str">
         <v>Zapit</v>
@@ -3263,7 +3263,7 @@
         <v>0.8</v>
       </c>
       <c r="AK22" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="AL22" t="str">
         <v>Zapit</v>
@@ -3397,7 +3397,7 @@
         <v>0.8</v>
       </c>
       <c r="AK23" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="AL23" t="str">
         <v>Zapit</v>
@@ -3665,7 +3665,7 @@
         <v>0.8</v>
       </c>
       <c r="AK25" t="str">
-        <v>TRUE</v>
+        <v>FALSE</v>
       </c>
       <c r="AL25" t="str">
         <v>Zapit</v>

</xml_diff>